<commit_message>
feat: harden Document AI labs for live delivery
</commit_message>
<xml_diff>
--- a/sample_docs/formats/quotation.xlsx
+++ b/sample_docs/formats/quotation.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="견적_요약" sheetId="1" r:id="R1b5f1ef8ec344a64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="품목" sheetId="2" r:id="R6dfd3b4b8fbd4edf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="형식_주의사항" sheetId="3" r:id="R3a4a3801df134de0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="견적_요약" sheetId="1" r:id="Rf33ac7034cfd4974"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="품목" sheetId="2" r:id="Rf3b99ed6e3eb47a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="형식_주의사항" sheetId="3" r:id="R4d1021dc2fab4a5e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -574,7 +574,7 @@
       <x:c r="C2" s="29" t="n">
         <x:v>85000</x:v>
       </x:c>
-      <x:c r="D2" s="22" t="n">
+      <x:c r="D2" s="29" t="n">
         <x:f>B2*C2</x:f>
         <x:v>340000</x:v>
       </x:c>
@@ -593,7 +593,7 @@
       <x:c r="C3" s="29" t="n">
         <x:v>160000</x:v>
       </x:c>
-      <x:c r="D3" s="22" t="n">
+      <x:c r="D3" s="29" t="n">
         <x:f>B3*C3</x:f>
         <x:v>160000</x:v>
       </x:c>
@@ -605,7 +605,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88982b064c564737"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa670b139abe4f67"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>